<commit_message>
Added Documentation and recording
</commit_message>
<xml_diff>
--- a/Test Cases Results.xlsx
+++ b/Test Cases Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nii-jraluib\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jraluib\AndroidStudioProjects\billease-appium-pom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42EFD9D-05CE-4EF8-BCB0-1912C793B925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C46284-31D3-4DB7-975B-0F9413540E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{EFF8BE47-2E32-48A2-8072-E126E883054A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EFF8BE47-2E32-48A2-8072-E126E883054A}"/>
   </bookViews>
   <sheets>
     <sheet name="Android_Login" sheetId="1" r:id="rId1"/>
@@ -1104,10 +1104,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
@@ -1136,9 +1136,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1176,7 +1176,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1282,7 +1282,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1424,7 +1424,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1433,18 +1433,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F571A4C0-E433-4AC5-B591-FD59CB289FAA}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.7109375" customWidth="1"/>
+    <col min="1" max="1" width="51.6640625" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="32.28515625" customWidth="1"/>
-    <col min="4" max="4" width="59.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" customWidth="1"/>
+    <col min="4" max="4" width="59.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="24.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>185</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>186</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>187</v>
       </c>
@@ -1533,7 +1533,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>188</v>
       </c>
@@ -1556,7 +1556,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>189</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>190</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>191</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>192</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>193</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>194</v>
       </c>
@@ -1696,18 +1696,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F0D6EC-CD12-4755-97D1-3D4F80421B4A}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.7109375" customWidth="1"/>
+    <col min="1" max="1" width="51.6640625" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="32.28515625" customWidth="1"/>
-    <col min="4" max="4" width="59.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" customWidth="1"/>
+    <col min="4" max="4" width="59.33203125" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>195</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>196</v>
       </c>
@@ -1773,7 +1773,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>197</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>198</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>199</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>200</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>201</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>202</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>203</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>204</v>
       </c>
@@ -1958,9 +1958,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{507D0FA4-B4A6-4100-90CD-1A3991252BC9}">
   <dimension ref="A1:G43"/>
-  <sheetFormatPr defaultColWidth="27.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="27.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="118.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>137</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>138</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>139</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>140</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>141</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>142</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>143</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>144</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>145</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>146</v>
       </c>
@@ -2183,14 +2183,14 @@
         <v>206</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B12" s="2"/>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>147</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>148</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>149</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>150</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>151</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>152</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>153</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>154</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>155</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>156</v>
       </c>
@@ -2420,7 +2420,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>94</v>
       </c>
@@ -2428,7 +2428,7 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>157</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>158</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>159</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>160</v>
       </c>
@@ -2520,7 +2520,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>161</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>162</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>163</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>164</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>165</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>166</v>
       </c>
@@ -2658,8 +2658,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>104</v>
       </c>
@@ -2667,7 +2667,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
     </row>
-    <row r="36" spans="1:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>167</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>168</v>
       </c>
@@ -2707,23 +2707,23 @@
         <v>206</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
     </row>
-    <row r="40" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="41" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
     </row>
-    <row r="42" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
     </row>
-    <row r="43" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -2741,13 +2741,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1C1E542-A93D-4356-B178-5901AC1278DB}">
   <dimension ref="A1:G37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="5" width="49.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="5" width="49.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>105</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>106</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>107</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>108</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>109</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>110</v>
       </c>
@@ -2890,7 +2890,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>111</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>112</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>113</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>114</v>
       </c>
@@ -2970,14 +2970,14 @@
         <v>206</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B12" s="2"/>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>115</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>116</v>
       </c>
@@ -3011,7 +3011,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>117</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>118</v>
       </c>
@@ -3039,7 +3039,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>119</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>120</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>121</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>122</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>123</v>
       </c>
@@ -3109,7 +3109,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>124</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>94</v>
       </c>
@@ -3131,7 +3131,7 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:4" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>125</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>126</v>
       </c>
@@ -3159,7 +3159,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>127</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>128</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>129</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>130</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>131</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>132</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>133</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>134</v>
       </c>
@@ -3271,8 +3271,8 @@
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="1:4" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>104</v>
       </c>
@@ -3280,7 +3280,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
     </row>
-    <row r="36" spans="1:4" ht="231.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>135</v>
       </c>
@@ -3291,7 +3291,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>136</v>
       </c>
@@ -3310,18 +3310,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAC3E569-5D80-4949-BB15-2372E7B30121}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
-    <col min="2" max="2" width="40.5703125" customWidth="1"/>
-    <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="4" width="36.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" customWidth="1"/>
+    <col min="2" max="2" width="40.5546875" customWidth="1"/>
+    <col min="3" max="3" width="29.88671875" customWidth="1"/>
+    <col min="4" max="4" width="36.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>284</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>285</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>286</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>287</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>288</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>289</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>290</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>291</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>292</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>293</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>294</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>295</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>296</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>297</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>298</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>299</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>300</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>301</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>302</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>303</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>304</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>305</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>306</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>307</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>308</v>
       </c>
@@ -3853,7 +3853,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>309</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>310</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>311</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>312</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>313</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>314</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>315</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>316</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>317</v>
       </c>
@@ -4045,18 +4045,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47A65F07-5205-407E-BE8E-BD966034A6BC}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="40.5703125" customWidth="1"/>
-    <col min="3" max="3" width="29.85546875" customWidth="1"/>
-    <col min="4" max="4" width="36.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" customWidth="1"/>
+    <col min="2" max="2" width="40.5546875" customWidth="1"/>
+    <col min="3" max="3" width="29.88671875" customWidth="1"/>
+    <col min="4" max="4" width="36.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>250</v>
       </c>
@@ -4099,7 +4099,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>251</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>252</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>253</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>254</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>266</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>267</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>268</v>
       </c>
@@ -4239,7 +4239,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>269</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>270</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>255</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>256</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>257</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>271</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>272</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>273</v>
       </c>
@@ -4408,7 +4408,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>274</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>275</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>258</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>276</v>
       </c>
@@ -4488,7 +4488,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>259</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>260</v>
       </c>
@@ -4528,7 +4528,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>261</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>277</v>
       </c>
@@ -4568,7 +4568,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>278</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>279</v>
       </c>
@@ -4608,7 +4608,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>280</v>
       </c>
@@ -4628,7 +4628,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>281</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>262</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>282</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>263</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>264</v>
       </c>
@@ -4728,7 +4728,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>265</v>
       </c>
@@ -4748,7 +4748,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>283</v>
       </c>

</xml_diff>